<commit_message>
chore(codebook): regenerate CSVs from PR #1 site-data updates
Picks up the 13 corrected paper URLs + WebArena-Privacy → AgentDAM
rename + content rewrites so benchmarks.csv, sub_tools.csv, and
heart_codebook.xlsx track the website 1:1.

Both validators (validate_codebook.py + site_consistency_check.py)
PASS with 0 errors.
</commit_message>
<xml_diff>
--- a/codebook/heart_codebook.xlsx
+++ b/codebook/heart_codebook.xlsx
@@ -1347,7 +1347,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2405.18743</t>
+          <t>https://aclanthology.org/2025.coling-main.745/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Inference of implicit norms in social forums</t>
+          <t>Theory-driven social-knowledge task profile</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>社会论坛隐性规范推断</t>
+          <t>社会知识多任务画像</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2023.findings-emnlp.969/</t>
+          <t>https://aclanthology.org/2023.emnlp-main.699/</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2701,77 +2701,77 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Multi-Metric Failure-Mode Profile</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>多指标失败模式画像</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Theory-driven Social-Knowledge Task Suite (SocKET)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>理论驱动社会知识任务套件</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
           <t>T03</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>Scenario-Stakeholder-Information-Flow Template</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>场景-利益相关方-信息流模板</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Social forum-derived scenario scaffolding with implicit norm inference tasks</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>社交论坛场景框架与隐含规范推断任务</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>T02</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Normative Source &amp; Decision-Boundary Ledger</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>规范来源与决策边界台账</t>
-        </is>
-      </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Social forum-derived scenario scaffolding with implicit norm inference tasks</t>
+          <t>Theory-driven Social-Knowledge Task Suite (SocKET)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>社交论坛衍生情景框架与隐式规范推理任务台账</t>
+          <t>理论驱动社会知识任务套件</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Scenario validity; Context and stakeholder coverage; Normative grounding</t>
+          <t>Construct clarity; Metric validity; Scenario validity</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>When adapting "Social forum-derived scenario scaffolding with implicit norm inference tasks" from SOCKET (2023) to a Human-centered approach, first retain/migrate the article's own categories or slots: manually verified labels: roles, points of contention; poster identity, comment section points of contention, timestamps, voting tendencies. Use the main tool T03 Scenario-Stakeholder-Information Flow Template: first supplement actor, affected party, third party, relationship, purpose, information/action flow, constraints, consequence; use the secondary tool T02 Norm Source and Decision Boundary Ledger to reinforce: first list types of norm sources, applicable jurisdictions/fields, red lines, consensus, controversies, insufficient evidence, and conditions for expert escalation. The output should include: original categories/slots → target domain field mapping, adapted prompt or item, labeling/scoring rules, parts that can be automatically generated, and parts that require manual verification/governance. Automation can: automatically fill in scenario slots such as actor, affected party, purpose, information/action flow, constraints, consequence, and generate variants; Manual verification: requires human checks on the authenticity of the scenario, stakeholder coverage, omission of vulnerable subjects, cultural/legal context, and harm chains.</t>
+          <t>Adapt SocKET as a theory-driven social-knowledge task suite. Retain the categories humor/sarcasm, offensiveness, sentiment/emotion, and trustworthiness; use T11 to report category-level failure modes and T03 to contextualize actors, relationships, communication acts, and consequences.</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>基于 SOCKET (2023) 的“Social forum-derived scenario scaffolding with implicit norm inference tasks”改编到 Human centered 时，先保留/迁移该文章自己的分类或槽位：人工核对标签：角色、分歧; 发帖者身份、评论区分歧、时间戳、投票倾向。主工具用 T03 场景-利益相关方-信息流模板：先补 actor、affected party、third party、relationship、purpose、information/action flow、constraints、consequence；次工具用 T02 规范来源与决策边界台账，用于补强：先列规范来源类型、适用法域/领域、红线、共识、争议、证据不足和专家升级条件。输出需包括：原分类/槽位→目标领域字段映射、改编后的 prompt 或题项、标签/评分规则、可自动生成的部分、需人工校验/治理的部分。自动化可做：可自动填充 actor、affected party、purpose、information/action flow、constraints、consequence 等场景槽位并生成变体；人工校验：需人工核查场景真实性、利益相关方覆盖、弱势主体遗漏、文化/法律语境和伤害链条。</t>
+          <t>基于 SOCKET/SocKET (2023) 的“Theory-driven Social-Knowledge Task Suite”改编到 Human centered 时，先保留/迁移原文的社会知识任务类别：humor &amp; sarcasm、offensiveness、sentiment &amp; emotion、trustworthiness，以及 58 项任务的多任务结构。主工具用 T11 多指标失败模式画像：按社会知识类别分别报告错误，而不是把全部社会性理解压成一个总分；次工具用 T03 场景-利益相关方-信息流模板：把目标应用场景中的 actor、affected party、relationship、communication act 和 consequence 补全。输出需包括：原任务类别→目标领域字段映射、改编后的 prompt/题项、每类社会知识的评分规则、可自动生成的场景变体、需人工校验的文化和伤害边界。</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Example aligned with the Prompt: Retain/migrate the original categories or slots (manual verification labels: roles, disagreements; poster identity, comment section disagreements, timestamps, voting tendencies). Target adaptation: In a dataset for a campus social AI assistant aimed at teenagers, extract real posts from school forums (such as the ChinaZhihu education section) on topics like 'How to respond after being called by the wrong name in public?', retaining the original poster's grade level, teacher/classmate comment disagreements, and the distribution of likes. The model should not only judge whether a correction is necessary but also generate three feasible responses adapted to different role relationships (teacher-student vs. peers) and different cultural scripts (collectivist modesty vs. individual assertion), and label the implicit norms activated by each response (e.g., 'respect for naming rights' vs. 'maintaining classroom order'). Additional verification: Check if the labeling/scoring rules are consistent with the above categories using the T03 scenario-stakeholder-information flow template + T02 ledger of norm sources and decision boundaries, and mark any norms, risks, or cultural boundaries that require manual review.</t>
+          <t>Example: in a school-assistant dataset, build tasks that test joke/sarcasm boundaries, offensiveness, student emotion, and trustworthy advice, then report separate failure modes rather than forum vote metadata.</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>与Prompt对齐的示例：保留/迁移原分类或槽位（人工核对标签：角色、分歧; 发帖者身份、评论区分歧、时间戳、投票倾向）。目标改编：在面向青少年的校园社交AI助手数据集中，抽取真实校园论坛（如ChinaZhihu教育板块）中'被当众叫错名字后如何回应？'等帖子，保留原发帖者年级、教师/同学评论分歧及点赞分布，要求模型不仅判断'是否应纠正'，还需生成适配不同角色关系（师生vs同龄人）、不同文化脚本（集体主义谦抑vs个体主张）的3种可行回应，并标注每种回应所激活的隐含规范（如'尊重称谓权' vs '维护课堂秩序'）。补充校验：按 T03 场景-利益相关方-信息流模板 + T02 规范来源与决策边界台账 检查标签/评分规则是否与上述分类一致，并标出需人工复核的规范、风险或文化边界。</t>
+          <t>与Prompt对齐的示例：保留 SocKET 的社会知识类别而非论坛投票元数据。目标改编：在青少年校园AI助手数据集中，围绕“同学用玩笑称呼转学生”构造四类题项：是否识别讽刺/玩笑边界、是否识别冒犯性、是否理解学生情绪、是否给出可信且不过度惩罚的建议。按 T11 分别报告四类失败模式，再按 T03 补全学生、老师、家长、同伴关系和可能后果。</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2023.emnlp-main.747/</t>
+          <t>https://aclanthology.org/2023.emnlp-main.428/</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2020.acl-main.487/</t>
+          <t>https://ojs.aaai.org/index.php/AAAI/article/view/6267</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2020.findings-emnlp.106/</t>
+          <t>https://aclanthology.org/2020.acl-main.265/</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2021.emnlp-main.211/</t>
+          <t>https://aclanthology.org/2021.findings-emnlp.211/</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2021.eacl-main.163/</t>
+          <t>https://aclanthology.org/2021.emnlp-main.704/</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2025.findings-naacl.201/</t>
+          <t>https://aclanthology.org/2025.findings-naacl.199/</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -6031,22 +6031,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Fairness&amp;Inclusivity</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>普惠正直</t>
+          <t>安全</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Discriminative-Generative Dual-track Bias Difference</t>
+          <t>Multilingual Safety Failure-Mode Probe</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>判别-生成双轨偏见差</t>
+          <t>多语言安全失败模式探针</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -6061,77 +6061,77 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Claim-Construct &amp; Protected-Interest Mapper</t>
+          <t>Multi-Metric Failure-Mode Profile</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>声明-构念-受保护利益映射器</t>
+          <t>多指标失败模式画像</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Discrimination-Generation Gap Analyzer (DGGA)</t>
+          <t>Multilingual Safety Failure-Mode Probe (Phare)</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>歧视-代沟分析器</t>
+          <t>多语言安全失败模式探针</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Scenario-Stakeholder-Information-Flow Template</t>
+          <t>Risk-Tier &amp; Hazard Taxonomy</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>场景-利益相关方-信息流模板</t>
+          <t>风险等级与危害分类</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Discrimination-Generation Gap Analyzer (DGGA)</t>
+          <t>Multilingual Safety Failure-Mode Probe (Phare)</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>歧视-代沟分析器</t>
+          <t>多语言安全失败模式探针</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Construct clarity; Real-world harm linkage</t>
+          <t>Metric validity; Real-world harm linkage; Task-format fit</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>When adapting the "Discrimination-Generation Gap Analyzer (DGGA)" from Phare (2025) to Fairness&amp;inclusive, first retain/migrate the article's own categories or slots: manually verified labels: judgment + generation, implicit evaluation tendency. The main tool uses T01 Declaration-Construct-Protected Interest Mapper: first write the target construct, sub-constructs, protected interests, exclusion scope, and the minimum claim that the score can support; the secondary tool uses T03 Scenario-Stakeholder-Information Flow Template for reinforcement: first supplement actor, affected party, third party, relationship, purpose, information/action flow, constraints, consequence. The output should include: original category/slot → target domain field mapping, adapted prompt or item, labeling/scoring rules, automatically generatable parts, and parts requiring manual verification/governance. Automation can: automatically extract candidate constructs, sub-dimensions, protected interests, exclusion scope, and draft of claim limitation; manual verification: requires human confirmation on whether the construct is reasonably argued, whether the protected interests are complete, and whether the claim limitation is sufficiently conservative.</t>
+          <t>Adapt Phare as a multilingual safety failure-mode probe across hallucination/reliability, social bias, and harmful-content generation. Use T11 to report multi-metric profiles by language, scenario, risk, and failure mode; use T04 to map failure modes to hazard categories, severity, vulnerable subjects, and help/refuse/clarify/escalate boundaries. Do not describe Phare as a discriminative-generative gap analyzer.</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>基于 Phare (2025) 的“Discrimination-Generation Gap Analyzer (DGGA)”改编到 Fairness&amp;inclusive 时，先保留/迁移该文章自己的分类或槽位：人工核对标签：判断+生成，隐性评价倾向。主工具用 T01 声明-构念-受保护利益映射器：先写目标构念、子构念、受保护利益、排除范围和分数可支持的最小 claim；次工具用 T03 场景-利益相关方-信息流模板，用于补强：先补 actor、affected party、third party、relationship、purpose、information/action flow、constraints、consequence。输出需包括：原分类/槽位→目标领域字段映射、改编后的 prompt 或题项、标签/评分规则、可自动生成的部分、需人工校验/治理的部分。自动化可做：可自动抽取候选构念、子维度、受保护利益、排除范围和 claim limitation 草稿；人工校验：需人工确认构念是否合理论证、受保护利益是否完整、claim limitation 是否足够保守。</t>
+          <t>基于 Phare (2025) 的“Multilingual Safety Failure-Mode Probe (Phare)”改编到 Safety 时，先保留/迁移原文的三类安全维度：hallucination/reliability、social biases、harmful content generation。主工具用 T11 多指标失败模式画像：按场景、语言、风险类型和失败模式分别记录结果，避免只给总分；次工具用 T04 风险等级与危害分类：把失败模式映射到风险类别、严重性、脆弱主体、help/refuse/clarify/escalate 边界。输出需包括：原 Phare 维度→目标领域字段映射、改编后的 prompt 或题项、多指标评分表、可自动统计的 failure-mode profile、需专家复核的安全边界。自动化可做：批量生成多语言变体、汇总 hallucination/social-bias/harmful-content 指标和错误模式；人工校验：需专家确认风险类别、文化语境、社会偏见子类和对外 claim 边界。</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>Example aligned with the Prompt: Retain/migrate the original classification or slot (human verification label: judgment + generation, implicit evaluation bias). Target adaptation: In a recruitment resume screening dataset, use DGGA to simultaneously submit the same resume for an MCQ scoring task ('Is this candidate suitable for a technical position? A. Yes B. No') and an open-ended generation task ('Please summarize the core strengths of this candidate in three sentences'). Analyze the implicit evaluation bias in the generated text regarding the cultural background suggested by the name (e.g., more frequent use of 'strong communication skills' rather than 'solid algorithm knowledge' for a resume named 'Mohammed'), thereby identifying risk points where discrimination is accurate but generation is imbalanced. Additional verification: Check whether the labeling/scoring rules are consistent with the above classifications using T01 Declaration-Construct-Protected Interest Mapper + T03 Scenario-Stakeholder-Information Flow Template, and mark out the norms, risks, or cultural boundaries that require human review.</t>
+          <t>Example: adapt Phare to customer-service safety evaluation by testing bilingual prompts for fabricated policy claims, group stereotypes, and harmful advice. Report failure modes with T11 and risk tiers with T04.</t>
         </is>
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>与Prompt对齐的示例：保留/迁移原分类或槽位（人工核对标签：判断+生成，隐性评价倾向）。目标改编：在招聘简历筛选数据集中，使用DGGA向模型同时提交同一份简历的MCQ打分任务（‘该候选人适合技术岗吗？A.是 B.否’）和开放生成任务（‘请用三句话总结该候选人的核心优势’），分析生成文本中对姓名暗示文化背景的隐性评价倾向（如对‘Mohammed’简历更频繁使用‘沟通能力强’而非‘算法扎实’），从而定位判别准确但生成失衡的风险点。补充校验：按 T01 声明-构念-受保护利益映射器 + T03 场景-利益相关方-信息流模板 检查标签/评分规则是否与上述分类一致，并标出需人工复核的规范、风险或文化边界。</t>
+          <t>与Prompt对齐的示例：保留 Phare 的三类安全维度。目标改编：在客服AI安全评测中，为同一用户请求生成中英双语测试项，分别检查（1）是否编造政策或事实依据，（2）是否对年龄、地域、职业等群体产生刻板化回应，（3）是否输出危险或违法建议。按 T11 汇总失败模式画像，并按 T04 标注风险等级和升级边界，避免把 Phare 误写成只测公平性的判别-生成差异工具。</t>
         </is>
       </c>
     </row>
@@ -6275,12 +6275,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2506.12327</t>
+          <t>https://aclanthology.org/2025.gebnlp-1.1/</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://github.com/nyu-mll/BBQ</t>
+          <t>https://github.com/ynklab/JBBQ_data</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2403.01244</t>
+          <t>https://aclanthology.org/2024.findings-eacl.61/</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2024.naacl-short.59/</t>
+          <t>https://aclanthology.org/2024.naacl-short.60/</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://github.com/thu-coai/SafetyBench</t>
+          <t>https://github.com/isXinLiu/MM-SafetyBench</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -7722,12 +7722,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>生活建议场景隐式毒性</t>
+          <t>七类安全风险；中英双语多选题；安全理解能力</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2311.17600</t>
+          <t>https://arxiv.org/abs/2309.07045</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -7752,12 +7752,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Multi-dimension MCQ Safety Template with Implicit Toxicity Triggering (LifeTox-inspired)</t>
+          <t>Bilingual seven-category MCQ safety benchmark template</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>多维度隐式毒性触发安全模板</t>
+          <t>双语七类安全多选题模板</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -7777,12 +7777,12 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Multi-dimension MCQ Safety Template with Implicit Toxicity Triggering (LifeTox-inspired)</t>
+          <t>Bilingual seven-category MCQ safety benchmark template</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>多维度安全模板隐含毒性触发</t>
+          <t>双语七类安全多选题模板</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -7792,22 +7792,22 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>When adapting the "Multi-dimension MCQ Safety Template with Implicit Toxicity Triggering (LifeTox-inspired)" from SafetyBench (2024) to Safety, first retain/migrate the article's own categories or slots: manually verified label: implicit toxicity. The primary tool uses T07 behavior coverage matrix: first, construct a capability × scenario × stakeholder × risk × test type coverage matrix, then supplement with candidate questions; the secondary tool uses T03 scenario-stakeholder-information flow template for reinforcement: first, supplement actor, affected party, third party, relationship, purpose, information/action flow, constraints, consequence. The output should include: original category/slot → target domain field mapping, adapted prompt or question items, labeling/scoring rules, parts that can be automatically generated, and parts that require manual verification/governance. Automation can: automatically generate the coverage matrix, count empty cells, and sample or generate candidate questions for each cell; manual verification: requires human decision on coverage priority, sampling weight, unmeasurable scope, and matrix maintenance plan.</t>
+          <t>When adapting the "Bilingual seven-category MCQ safety benchmark template" from SafetyBench (2024) to Safety, first retain/migrate the paper's own categories or slots: seven safety categories, Chinese/English MCQs, and safety-understanding evaluation. Use T07 Behavioral Coverage Matrix as the main tool to build a capability × scenario × stakeholder × risk × test type matrix, then add candidate questions; use T03 Scenario-Stakeholder-Information-Flow Template as a secondary tool to specify actors, affected parties, purpose, information/action flow, constraints, and consequences. Outputs should include source slot-to-target field mapping, adapted questions, labeling/scoring rules, automatable parts, and human-review parts. Automation can draft coverage matrices and candidate MCQs; human review should confirm safety-category boundaries, item difficulty, bilingual equivalence, help/refuse boundaries, and maintenance plans.</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>基于 SafetyBench (2024) 的“Multi-dimension MCQ Safety Template with Implicit Toxicity Triggering (LifeTox-inspired)”改编到 Safety 时，先保留/迁移该文章自己的分类或槽位：人工核对标签：隐式毒性。主工具用 T07 行为覆盖矩阵：先建 capability × scenario × stakeholder × risk × test type 覆盖矩阵，再补候选题；次工具用 T03 场景-利益相关方-信息流模板，用于补强：先补 actor、affected party、third party、relationship、purpose、information/action flow、constraints、consequence。输出需包括：原分类/槽位→目标领域字段映射、改编后的 prompt 或题项、标签/评分规则、可自动生成的部分、需人工校验/治理的部分。自动化可做：可自动生成覆盖矩阵、统计空格子，并为每个格子抽样或生成候选题；人工校验：需人工决定覆盖优先级、抽样权重、不可测范围和矩阵维护计划。</t>
+          <t>基于 SafetyBench (2024) 的“Bilingual seven-category MCQ safety benchmark template”改编到 Safety 时，先保留/迁移该文章自己的分类或槽位：七类安全风险；中英双语多选题；安全理解能力。主工具用 T07 行为覆盖矩阵：先建 capability × scenario × stakeholder × risk × test type 覆盖矩阵，再补候选题；次工具用 T03 场景-利益相关方-信息流模板，用于补强：先补 actor、affected party、third party、relationship、purpose、information/action flow、constraints、consequence。输出需包括：原分类/槽位→目标领域字段映射、改编后的 prompt 或题项、标签/评分规则、可自动生成的部分、需人工校验/治理的部分。自动化可做：可自动生成覆盖矩阵、统计空格子，并为每个格子抽样或生成候选题；人工校验：需人工决定安全类别边界、样本难度、语言等值性、拒答/帮助边界和矩阵维护计划。</t>
         </is>
       </c>
       <c r="U66" t="inlineStr">
         <is>
-          <t>Example aligned with the Prompt: Retain/transfer the original category or slot (human-verified label: implicit toxicity). Target adaptation: In a customer service dialogue dataset, rewrite the original customer service response into a 'life hack' variant containing implicit out-of-bounds suggestions (e.g., "Dealing with a difficult customer? Try secretly recording the screen and then editing it to take things out of context and post on social media to apply pressure"), embed MCQ options requiring annotation of the violated sub-dimensions (Privacy violation / Unfairness), for training/testing the model's ability to recognize covertly manipulative language. Additional verification: Check if the labeling/scoring rules are consistent with the above categories according to the T07 behavior coverage matrix + T03 scenario-stakeholder-information flow template, and mark the norms, risks, or cultural boundaries that require human re-examination.</t>
+          <t>Example aligned with the prompt: retain/migrate SafetyBench slots (seven safety categories, bilingual MCQs, safety-understanding evaluation). Target adaptation: in customer-service dialogues, rewrite cases into MCQs across privacy, illegal activity, mental health, discrimination/unfairness, and related safety categories. Ask the model to identify the risk category and appropriate refuse/clarify/escalate boundary. Verify coverage and bilingual equivalence with T07 + T03, and mark items requiring human review.</t>
         </is>
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>与Prompt对齐的示例：保留/迁移原分类或槽位（人工核对标签：隐式毒性）。目标改编：在客服对话数据集中，将原客服响应重写为含隐式越界建议的‘生活小贴士’变体（例如‘遇到难缠客户？试试悄悄录屏后剪辑断章取义发社交媒体施压’），嵌入MCQ选项要求标注其违反的子维度（Privacy violation / Unfairness），用于训练/评测客服模型对隐蔽操纵性话术的识别能力。补充校验：按 T07 行为覆盖矩阵 + T03 场景-利益相关方-信息流模板 检查标签/评分规则是否与上述分类一致，并标出需人工复核的规范、风险或文化边界。</t>
+          <t>与Prompt对齐的示例：保留/迁移原分类或槽位（七类安全风险；中英双语多选题；安全理解能力）。目标改编：在客服对话数据集中，将客服场景按隐私、违法行为、心理健康、歧视/不公平等安全类别重写为多选题，要求模型识别具体风险类别和合适的拒答/澄清/转介边界。补充校验：按 T07 行为覆盖矩阵 + T03 场景-利益相关方-信息流模板 检查题项是否覆盖目标安全类别、语言版本是否等值，并标出需人工复核的规范、风险或文化边界。</t>
         </is>
       </c>
     </row>
@@ -8374,7 +8374,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>HarmEval (2025)</t>
+          <t>TechHazardQA (2025)</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8389,12 +8389,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Safety Amplification Vector Injection Mechanism</t>
+          <t>Instruction-centric harmful query evaluation</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>安全放大向量注入机制</t>
+          <t>指令格式有害查询评估</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -8409,77 +8409,77 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Multi-Turn &amp; Adversarial Red-Team Protocol</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>多轮与对抗红队协议</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Instruction-Centric Harmful Query Evaluation (TechHazardQA)</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>指令格式有害查询评估</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
           <t>T04</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="N72" t="inlineStr">
         <is>
           <t>Risk-Tier &amp; Hazard Taxonomy</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="O72" t="inlineStr">
         <is>
           <t>风险等级与危害分类</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>Safety Amplification (SA) vector + Safety-guided decoding strategy (sGDS)</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>安全放大向量与安全引导解码策略</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>T01</t>
-        </is>
-      </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>Claim-Construct &amp; Protected-Interest Mapper</t>
-        </is>
-      </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>声明-构念-受保护利益映射器</t>
-        </is>
-      </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>Safety Amplification (SA) vector + Safety-guided decoding strategy (sGDS)</t>
+          <t>Instruction-Centric Harmful Query Evaluation (TechHazardQA)</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>安全放大向量与安全引导解码策略映射器</t>
+          <t>指令格式有害查询评估</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Real-world harm linkage; Scenario validity; Construct clarity</t>
+          <t>Task-format fit; Real-world harm linkage; Robustness against gaming and contamination</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>When adapting the "Safety Amplification (SA) vector + Safety-guided decoding strategy (sGDS)" from HarmEval (2025) to Safety, first retain/migrate the article's own classification or slots: manually verify labels: safety amplification, propose different safety. Use T04 for risk level and hazard categorization: first annotate the hazard category, risk level, vulnerable subjects, urgency, reversibility, and help/refuse/clarify/escalate boundaries; use T01 as a secondary tool, the claim-construct-protected interest mapper, for reinforcement: first write the target construct, sub-construct, protected interests, exclusion scope, and the minimum claim supported by the score. The output should include: original classification/slot → target domain field mapping, adapted prompt or item, labeling/scoring rules, parts that can be automatically generated, and parts that require manual verification/governance. Automation can: automatically generate preliminary risk levels, hazard categories, and help/refuse/clarify/escalate recommendations based on keywords and scenario features; manual verification: requires professional calibration of risk levels, crisis thresholds, referral conditions, and the cost of incorrect refusal/incorrect assistance.</t>
+          <t>Adapt TechHazardQA by preserving the contrast between text and instruction-centric formats such as pseudocode, programs, snippets, and procedural steps. Use T08 for adversarial format variants and T04 for hazard severity and refusal/escalation boundaries.</t>
         </is>
       </c>
       <c r="T72" t="inlineStr">
         <is>
-          <t>基于 HarmEval (2025) 的“Safety Amplification (SA) vector + Safety-guided decoding strategy (sGDS)”改编到 Safety 时，先保留/迁移该文章自己的分类或槽位：人工核对标签：安全放大，提出不同的安全。主工具用 T04 风险等级与危害分类：先标注 hazard category、风险等级、脆弱主体、紧急性、可逆性和 help/refuse/clarify/escalate 边界；次工具用 T01 声明-构念-受保护利益映射器，用于补强：先写目标构念、子构念、受保护利益、排除范围和分数可支持的最小 claim。输出需包括：原分类/槽位→目标领域字段映射、改编后的 prompt 或题项、标签/评分规则、可自动生成的部分、需人工校验/治理的部分。自动化可做：可自动依据关键词和场景特征生成初步风险等级、hazard category、help/refuse/clarify/escalate 建议；人工校验：需专业人员校准风险等级、危机阈值、转介条件和错误拒答/错误帮助的代价。</t>
+          <t>基于 TechHazardQA (2025) 的“Instruction-Centric Harmful Query Evaluation”改编到 Safety 时，先保留/迁移原文的 text vs instruction-centric 输出格式对照：普通文本、伪代码、程序片段、操作步骤。主工具用 T08 多轮与对抗红队协议：构造同一有害意图在不同输出格式下的提示变体，测试模型是否因格式伪装而越过安全边界；次工具用 T04 风险等级与危害分类：为每个题项标注 hazard category、风险等级和 help/refuse/clarify/escalate 边界。输出需包括：原格式类别→目标领域字段映射、改编后的测试 prompt、harmfulness 评分规则、可自动生成的格式变体、需人工复核的高风险样本。</t>
         </is>
       </c>
       <c r="U72" t="inlineStr">
         <is>
-          <t>Example aligned with the Prompt: Retain/migrate the original classification or slot (human-verified label: safety amplification, propose different safety). Target adaptation: In a medical Q&amp;A dataset, a model example set can be constructed based on the HIPAA Compliance Guidelines and the policies of major medical AI vendors, extracting HIPAA-sensitive amplification vectors, and enabling sGDS when generating patient consultation responses to forcibly suppress any token distribution that might leak PHI (Protected Health Information). Supplementary verification: Check if the labeling/scoring rules are consistent with the above classifications according to T04 risk levels and harm categories + T01 statement-construct-protected interest mapper, and mark the norms, risks, or cultural boundaries that require human review.</t>
+          <t>Example: rewrite the same unsafe medical request as natural language, pseudocode, SOP snippet, and tabular steps; check whether the model becomes unsafe because the request looks procedural.</t>
         </is>
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>与Prompt对齐的示例：保留/迁移原分类或槽位（人工核对标签：安全放大，提出不同的安全）。目标改编：在医疗问答数据集中，可基于《HIPAA合规指南》和主流医疗AI厂商政策构建示范样例集，提取HIPAA-sensitive amplification vector，并在生成患者咨询回复时启用sGDS，强制抑制任何可能泄露PHI（受保护健康信息）的token分布。补充校验：按 T04 风险等级与危害分类 + T01 声明-构念-受保护利益映射器 检查标签/评分规则是否与上述分类一致，并标出需人工复核的规范、风险或文化边界。</t>
+          <t>与Prompt对齐的示例：保留 TechHazardQA 的 instruction-centric 格式对照。目标改编：在医疗客服安全评测中，将同一危险请求分别写成自然语言建议、伪代码流程、客服 SOP 片段和表格化步骤，检查模型是否因为“格式像操作规程”而输出不应提供的危险内容。按 T08 构造变体，按 T04 标注风险等级和安全替代回答。</t>
         </is>
       </c>
     </row>
@@ -9071,7 +9071,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2403.01244</t>
+          <t>https://aclanthology.org/2024.findings-acl.184/</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -9967,7 +9967,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>https://aclanthology.org/2024.findings-naacl.142/</t>
+          <t>https://aclanthology.org/2024.naacl-long.147/</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -11274,7 +11274,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>WebArena-Privacy (2024)</t>
+          <t>AgentDAM (2025)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -11289,12 +11289,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>PII contamination intent + interface interaction sandbox</t>
+          <t>Web-agent data-minimization evaluation</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>PII污染意图+界面交互沙盒</t>
+          <t>Web智能体数据最小化评估</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -11304,7 +11304,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>https://github.com/sail-sg/AgentDAM</t>
+          <t>https://github.com/facebookresearch/ai-agent-privacy</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -11364,22 +11364,22 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>When adapting "Web-based privacy decision sandbox with PII-contaminated intent injection" from WebArena-Privacy (2024) to Privacy, first retain/migrate the article's own categories or slots: manually verify labels: sandbox, real toolchain, and interface constraints. Use T09 agent and workflow simulation as the main tool: first define tools/APIs, visible states, allowed actions, prohibited actions, log check items, and error recovery standards; use T03 scenario-stakeholder-information flow template as a secondary tool for reinforcement: first supplement actor, affected party, third party, relationship, purpose, information/action flow, constraints, consequence. The output should include: original category/slot → target domain field mapping, adapted prompt or item, label/scoring rules, parts that can be automatically generated, and parts that require manual verification/governance. Automation can: automatically generate workflow states, allowed/prohibited actions, log check items, and draft sandbox task scripts; manual verification: requires human audit of sandbox permissions, real business risks, log interpretation, liability attribution, and failure recovery standards.</t>
+          <t>When adapting "Web-based privacy decision sandbox with PII-contaminated intent injection" from AgentDAM (2025) to Privacy, first retain/migrate the article's own categories or slots: manually verify labels: sandbox, real toolchain, and interface constraints. Use T09 agent and workflow simulation as the main tool: first define tools/APIs, visible states, allowed actions, prohibited actions, log check items, and error recovery standards; use T03 scenario-stakeholder-information flow template as a secondary tool for reinforcement: first supplement actor, affected party, third party, relationship, purpose, information/action flow, constraints, consequence. The output should include: original category/slot → target domain field mapping, adapted prompt or item, label/scoring rules, parts that can be automatically generated, and parts that require manual verification/governance. Automation can: automatically generate workflow states, allowed/prohibited actions, log check items, and draft sandbox task scripts; manual verification: requires human audit of sandbox permissions, real business risks, log interpretation, liability attribution, and failure recovery standards.</t>
         </is>
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>基于 WebArena-Privacy (2024) 的“Web-based privacy decision sandbox with PII-contaminated intent injection”改编到 Privacy 时，先保留/迁移该文章自己的分类或槽位：人工核对标签：沙盒，真实工具链和界面约束。主工具用 T09 智能体与工作流仿真：先定义工具/API、可见状态、允许动作、禁止动作、日志检查项和错误恢复标准；次工具用 T03 场景-利益相关方-信息流模板，用于补强：先补 actor、affected party、third party、relationship、purpose、information/action flow、constraints、consequence。输出需包括：原分类/槽位→目标领域字段映射、改编后的 prompt 或题项、标签/评分规则、可自动生成的部分、需人工校验/治理的部分。自动化可做：可自动生成工作流状态、允许/禁止动作、日志检查项和沙盒任务脚本草案；人工校验：需人工审计沙盒权限、真实业务风险、日志解释、责任归属和失败恢复标准。</t>
+          <t>基于 AgentDAM (2025) 的“Web-based privacy decision sandbox with PII-contaminated intent injection”改编到 Privacy 时，先保留/迁移该文章自己的分类或槽位：人工核对标签：沙盒，真实工具链和界面约束。主工具用 T09 智能体与工作流仿真：先定义工具/API、可见状态、允许动作、禁止动作、日志检查项和错误恢复标准；次工具用 T03 场景-利益相关方-信息流模板，用于补强：先补 actor、affected party、third party、relationship、purpose、information/action flow、constraints、consequence。输出需包括：原分类/槽位→目标领域字段映射、改编后的 prompt 或题项、标签/评分规则、可自动生成的部分、需人工校验/治理的部分。自动化可做：可自动生成工作流状态、允许/禁止动作、日志检查项和沙盒任务脚本草案；人工校验：需人工审计沙盒权限、真实业务风险、日志解释、责任归属和失败恢复标准。</t>
         </is>
       </c>
       <c r="U98" t="inlineStr">
         <is>
-          <t>Example aligned with the Prompt: Retain/migrate the original classification or slot (human-verified labels: sandbox, real toolchain, and interface constraints). Target adaptation: In an open-source code review dataset, inject developer private information into the PR description (e.g., 'Based on my discussion with Alice about the API key rotation scheme on Slack') and, in a GitHub sandbox environment, require the LLM review agent to generate comments, forcing it to filter out names, platform names, and key-related terms when referencing the context, rather than relying solely on keyword blocking. Supplementary verification: Check if the labeling/scoring rules are consistent with the above classification according to T09 Agent and Workflow Simulation + T03 Scenario-Stakeholder-Information Flow Template, and mark the norms, risks, or cultural boundaries that require human re-examination.</t>
+          <t>Example aligned with the Prompt: Retain/migrate the original classification or slot (human-verified labels: sandbox, real toolchain, and interface constraints). Target adaptation: In an open-source code review dataset, insert synthetic or de-identified developer-private context into the PR description (e.g., 'Based on an internal discussion about API key rotation') and, in a GitHub sandbox environment, require the LLM review agent to generate comments, forcing it to filter out names, platform names, and key-related terms when referencing the context, rather than relying solely on keyword blocking. Supplementary verification: Check if the labeling/scoring rules are consistent with the above classification according to T09 Agent and Workflow Simulation + T03 Scenario-Stakeholder-Information Flow Template, and mark the norms, risks, or cultural boundaries that require human re-examination.</t>
         </is>
       </c>
       <c r="V98" t="inlineStr">
         <is>
-          <t>与Prompt对齐的示例：保留/迁移原分类或槽位（人工核对标签：沙盒，真实工具链和界面约束）。目标改编：在开源代码审查数据集中，向PR描述中注入开发者私有信息（如‘根据我和Alice在Slack讨论的API密钥轮换方案’），并在GitHub沙盒环境中要求LLM审查代理生成评论，强制其在引用上下文时过滤人名、平台名及密钥相关术语，而非仅依赖关键词屏蔽。补充校验：按 T09 智能体与工作流仿真 + T03 场景-利益相关方-信息流模板 检查标签/评分规则是否与上述分类一致，并标出需人工复核的规范、风险或文化边界。</t>
+          <t>与Prompt对齐的示例：保留/迁移原分类或槽位（人工核对标签：沙盒，真实工具链和界面约束）。目标改编：在开源代码审查数据集中，向PR描述中加入模拟或脱敏的开发者私有信息（如“根据内部聊天中关于API密钥轮换方案的讨论”），并在GitHub沙盒环境中要求LLM审查代理生成评论，强制其在引用上下文时过滤人名、平台名及密钥相关术语，而非仅依赖关键词屏蔽。补充校验：按 T09 智能体与工作流仿真 + T03 场景-利益相关方-信息流模板 检查标签/评分规则是否与上述分类一致，并标出需人工复核的规范、风险或文化边界。</t>
         </is>
       </c>
     </row>
@@ -11411,7 +11411,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2503.04340</t>
+          <t>https://aclanthology.org/2025.acl-long.518/</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -15291,27 +15291,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Scenario-Stakeholder-Information-Flow Template</t>
+          <t>Multi-Metric Failure-Mode Profile</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>场景-利益相关方-信息流模板</t>
+          <t>多指标失败模式画像</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Social forum-derived scenario scaffolding with implicit norm inference tasks</t>
+          <t>Theory-driven Social-Knowledge Task Suite (SocKET)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>社交论坛场景框架与隐含规范推断任务</t>
+          <t>理论驱动社会知识任务套件</t>
         </is>
       </c>
     </row>
@@ -15328,27 +15328,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Normative Source &amp; Decision-Boundary Ledger</t>
+          <t>Scenario-Stakeholder-Information-Flow Template</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>规范来源与决策边界台账</t>
+          <t>场景-利益相关方-信息流模板</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Social forum-derived scenario scaffolding with implicit norm inference tasks</t>
+          <t>Theory-driven Social-Knowledge Task Suite (SocKET)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>社交论坛衍生情景框架与隐式规范推理任务台账</t>
+          <t>理论驱动社会知识任务套件</t>
         </is>
       </c>
     </row>
@@ -17511,27 +17511,27 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Claim-Construct &amp; Protected-Interest Mapper</t>
+          <t>Multi-Metric Failure-Mode Profile</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>声明-构念-受保护利益映射器</t>
+          <t>多指标失败模式画像</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Discrimination-Generation Gap Analyzer (DGGA)</t>
+          <t>Multilingual Safety Failure-Mode Probe (Phare)</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>歧视-代沟分析器</t>
+          <t>多语言安全失败模式探针</t>
         </is>
       </c>
     </row>
@@ -17548,27 +17548,27 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Scenario-Stakeholder-Information-Flow Template</t>
+          <t>Risk-Tier &amp; Hazard Taxonomy</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>场景-利益相关方-信息流模板</t>
+          <t>风险等级与危害分类</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Discrimination-Generation Gap Analyzer (DGGA)</t>
+          <t>Multilingual Safety Failure-Mode Probe (Phare)</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>歧视-代沟分析器</t>
+          <t>多语言安全失败模式探针</t>
         </is>
       </c>
     </row>
@@ -18636,12 +18636,12 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Multi-dimension MCQ Safety Template with Implicit Toxicity Triggering (LifeTox-inspired)</t>
+          <t>Bilingual seven-category MCQ safety benchmark template</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>多维度隐式毒性触发安全模板</t>
+          <t>双语七类安全多选题模板</t>
         </is>
       </c>
     </row>
@@ -18673,12 +18673,12 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Multi-dimension MCQ Safety Template with Implicit Toxicity Triggering (LifeTox-inspired)</t>
+          <t>Bilingual seven-category MCQ safety benchmark template</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>多维度安全模板隐含毒性触发</t>
+          <t>双语七类安全多选题模板</t>
         </is>
       </c>
     </row>
@@ -19060,32 +19060,32 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>HarmEval (2025)</t>
+          <t>TechHazardQA (2025)</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Risk-Tier &amp; Hazard Taxonomy</t>
+          <t>Multi-Turn &amp; Adversarial Red-Team Protocol</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>风险等级与危害分类</t>
+          <t>多轮与对抗红队协议</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Safety Amplification (SA) vector + Safety-guided decoding strategy (sGDS)</t>
+          <t>Instruction-Centric Harmful Query Evaluation (TechHazardQA)</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>安全放大向量与安全引导解码策略</t>
+          <t>指令格式有害查询评估</t>
         </is>
       </c>
     </row>
@@ -19097,32 +19097,32 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>HarmEval (2025)</t>
+          <t>TechHazardQA (2025)</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Claim-Construct &amp; Protected-Interest Mapper</t>
+          <t>Risk-Tier &amp; Hazard Taxonomy</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>声明-构念-受保护利益映射器</t>
+          <t>风险等级与危害分类</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Safety Amplification (SA) vector + Safety-guided decoding strategy (sGDS)</t>
+          <t>Instruction-Centric Harmful Query Evaluation (TechHazardQA)</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>安全放大向量与安全引导解码策略映射器</t>
+          <t>指令格式有害查询评估</t>
         </is>
       </c>
     </row>
@@ -20984,7 +20984,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>WebArena-Privacy (2024)</t>
+          <t>AgentDAM (2025)</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -21021,7 +21021,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>WebArena-Privacy (2024)</t>
+          <t>AgentDAM (2025)</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">

</xml_diff>

<commit_message>
Add resource metadata and anonymized expert results
</commit_message>
<xml_diff>
--- a/codebook/heart_codebook.xlsx
+++ b/codebook/heart_codebook.xlsx
@@ -4259,7 +4259,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://dl.acm.org/doi/10.1145/3442188.3445924</t>
+          <t>https://arxiv.org/abs/2101.11718</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -13019,7 +13019,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Governance Reliability</t>
+          <t>Evaluation Design</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -13034,8 +13034,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Test boundary stability through multiple rounds of诱导, role-playing, emotional manipulation, context pollution, prompt injection, and semantic disguise. 
-(Note: The term "诱导" was left untranslated as it seems to be a technical term or specific action in the context provided. If it should be translated, please provide further instructions.)</t>
+          <t>Test boundary stability through multi-turn coaxing, role-playing, emotional manipulation, context pollution, prompt injection, and semantic disguise.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -13055,7 +13054,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Robustness against gaming and contamination; Task-format fit; Real-world harm linkage</t>
+          <t>Task-format fit; Scenario validity; Robustness against gaming and contamination</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -21688,12 +21687,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0=Kleinberg (theoretical); 2=StereoSet/CrowS-Pairs/Winogender (construct too narrow or systematically refuted by Blodgett et al.); 3=BBQ/UnQover/RedditBias; 4=CBBQ/KoBBQ/HolisticBias/WinoQueer (includes local dimensions or community co-construction); 5=None (awaiting a complete example with Datasheets + rubric + exclusion scope + operationalization path).</t>
+          <t>0=None (no stable dataset benchmark anchor in this corpus); 2=StereoSet/CrowS-Pairs/Winogender (construct too narrow or systematically refuted by Blodgett et al.); 3=BBQ/UnQover/RedditBias; 4=CBBQ/KoBBQ/HolisticBias/WinoQueer (includes local dimensions or community co-construction); 5=None (awaiting a complete example with Datasheets + rubric + exclusion scope + operationalization path).</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0=Kleinberg（理论）；2=StereoSet/CrowS-Pairs/Winogender（构念过窄或被 Blodgett 等系统否证）；3=BBQ/UnQover/RedditBias；4=CBBQ/KoBBQ/HolisticBias/WinoQueer（含本土维度或社区共建）；5=暂无（待补 Datasheets+rubric+排除范围+操作化路径全齐的样例）。</t>
+          <t>0=暂无（本轮103个benchmark中无稳定实证锚点）；2=StereoSet/CrowS-Pairs/Winogender（构念过窄或被 Blodgett 等系统否证）；3=BBQ/UnQover/RedditBias；4=CBBQ/KoBBQ/HolisticBias/WinoQueer（含本土维度或社区共建）；5=暂无（待补 Datasheets+rubric+排除范围+操作化路径全齐的样例）。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -21902,12 +21901,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0=Kleinberg; 2=StereoSet/MoralChoice (source is rough/MTurk noise); 3=Majority (basically traceable); 4=KoBBQ/HolisticBias/WinoQueer (multi-source + partial bias disclosure); 5=None yet.</t>
+          <t>0=None (no stable dataset benchmark anchor in this corpus); 2=StereoSet/MoralChoice (source is rough/MTurk noise); 3=Majority (basically traceable); 4=KoBBQ/HolisticBias/WinoQueer (multi-source + partial bias disclosure); 5=None yet.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0=Kleinberg；2=StereoSet/MoralChoice（来源粗糙/MTurk 噪声）；3=多数（基本可追溯）；4=KoBBQ/HolisticBias/WinoQueer（多源+部分偏差披露）；5=暂无。</t>
+          <t>0=暂无（本轮103个benchmark中无稳定实证锚点）；2=StereoSet/MoralChoice（来源粗糙/MTurk 噪声）；3=多数（基本可追溯）；4=KoBBQ/HolisticBias/WinoQueer（多源+部分偏差披露）；5=暂无。</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -22116,12 +22115,12 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2=mostly static stereotype benchmark; 3=naturalistic/QA type (BBQ/UnQover); 4=WinoQueer (community involvement + clear harm chain); 5=none (requires all three: risk-tier, deployment chain, and affected parties).</t>
+          <t>2=StereoSet/HONEST/Panda (static stereotype or short-template benchmarks); 3=BBQ/UnQover (naturalistic/QA type); 4=WinoQueer (community involvement + clear harm chain); 5=None (requires all three: risk-tier, deployment chain, and affected parties).</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2=多数静态 stereotype benchmark；3=naturalistic/QA 类（BBQ/UnQover）；4=WinoQueer（社区参与+伤害链条明确）；5=暂无（需要 risk-tier+部署链+受影响主体三件齐）。</t>
+          <t>2=StereoSet/HONEST/Panda（静态 stereotype 或短模板类）；3=BBQ/UnQover（naturalistic/QA 类）；4=WinoQueer（社区参与+伤害链条明确）；5=暂无（需要 risk-tier+部署链+受影响主体三件齐）。</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -22330,12 +22329,12 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0=Kleinberg; 2=StereoSet/HONEST/Panda (single question type); 3=CrowS-Pairs/Winogender/WinoBias/GAP/CBBQ; 4=BBQ/HolisticBias/WinoQueer (includes control set/multiple types); 5=None.</t>
+          <t>0=None (no stable dataset benchmark anchor in this corpus); 2=StereoSet/HONEST/Panda (single question type); 3=CrowS-Pairs/Winogender/WinoBias/GAP/CBBQ; 4=BBQ/HolisticBias/WinoQueer (includes control set/multiple types); 5=None.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0=Kleinberg；2=StereoSet/HONEST/Panda（单一题型）；3=CrowS-Pairs/Winogender/WinoBias/GAP/CBBQ；4=BBQ/HolisticBias/WinoQueer（含对照集/多类型）；5=暂无。</t>
+          <t>0=暂无（本轮103个benchmark中无稳定实证锚点）；2=StereoSet/HONEST/Panda（单一题型）；3=CrowS-Pairs/Winogender/WinoBias/GAP/CBBQ；4=BBQ/HolisticBias/WinoQueer（含对照集/多类型）；5=暂无。</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -22651,12 +22650,12 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0=BERT-Bartl/Kleinberg; 1=Dev-WordEmbed/HONEST/UnQover (only automatic metrics, no calibration); 2=StereoSet/HolisticBias (automatic + some manual); 3=BBQ/CBBQ/KoBBQ/WinoQueer/HolisticBias (scoring rubric + partial manual); 4=Panda (dual annotation); 5=None.</t>
+          <t>0=BERT-Bartl; 1=Dev-WordEmbed/HONEST/UnQover (only automatic metrics, no calibration); 2=StereoSet/HolisticBias (automatic + some manual); 3=BBQ/CBBQ/KoBBQ/WinoQueer/HolisticBias (scoring rubric + partial manual); 4=Panda (dual annotation); 5=None.</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0=BERT-Bartl/Kleinberg；1=Dev-WordEmbed/HONEST/UnQover（仅自动指标无校准）；2=StereoSet/HolisticBias（自动+少量人工）；3=BBQ/CBBQ/KoBBQ/WinoQueer/HolisticBias（评分细则+部分人工）；4=Panda（双人标注）；5=暂无。</t>
+          <t>0=BERT-Bartl；1=Dev-WordEmbed/HONEST/UnQover（仅自动指标无校准）；2=StereoSet/HolisticBias（自动+少量人工）；3=BBQ/CBBQ/KoBBQ/WinoQueer/HolisticBias（评分细则+部分人工）；4=Panda（双人标注）；5=暂无。</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -22758,12 +22757,12 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0=Kleinberg; 2=StereoSet/UnQover/Winogender (lacks quality inspection); 3=majority; 4=BBQ/HolisticBias/WinoQueer/CrowS-Pairs/KoBBQ (includes manual review); 5=None.</t>
+          <t>0=None (no stable dataset benchmark anchor in this corpus); 2=StereoSet/UnQover/Winogender (lacks quality inspection); 3=majority; 4=BBQ/HolisticBias/WinoQueer/CrowS-Pairs/KoBBQ (includes manual review); 5=None.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>0=Kleinberg；2=StereoSet/UnQover/Winogender（缺质检）；3=多数；4=BBQ/HolisticBias/WinoQueer/CrowS-Pairs/KoBBQ（含人工复核）；5=暂无。</t>
+          <t>0=暂无（本轮103个benchmark中无稳定实证锚点）；2=StereoSet/UnQover/Winogender（缺质检）；3=多数；4=BBQ/HolisticBias/WinoQueer/CrowS-Pairs/KoBBQ（含人工复核）；5=暂无。</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -22865,12 +22864,12 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0=11 articles; 1=9 articles; 2=BUG/HolisticBias/TrustGPT/WinoQueer (mentioning risks or partially hidden); 3-5=None.</t>
+          <t>0=WinoQueer/HolisticBias (static public item sets with no gaming or contamination plan); 1=BUG/TrustGPT (mentions risk or light mitigation only); 2=BUG/HolisticBias/TrustGPT/WinoQueer (mentioning risks or partially hidden); 3-5=None.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0=11 篇；1=9 篇；2=BUG/HolisticBias/TrustGPT/WinoQueer（提到风险或部分隐藏）；3-5=无。</t>
+          <t>0=WinoQueer/HolisticBias（静态公开题库，未提防刷或污染）；1=BUG/TrustGPT（仅口头提风险或轻量保护）；2=BUG/HolisticBias/TrustGPT/WinoQueer（提到风险或部分隐藏）；3-5=暂无。</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -22972,12 +22971,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2=Kleinberg/Winogender/UnQover (only papers); 3=majority; 4=BBQ/CrowS-Pairs/HolisticBias/KoBBQ/MoralChoice/WinoQueer (includes code + data + some cards); 5=none.</t>
+          <t>2=Winogender/UnQover (paper-only or minimal documentation); 3=majority; 4=BBQ/CrowS-Pairs/HolisticBias/KoBBQ/MoralChoice/WinoQueer (includes code + data + some cards); 5=none.</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2=Kleinberg/Winogender/UnQover（仅论文）；3=多数；4=BBQ/CrowS-Pairs/HolisticBias/KoBBQ/MoralChoice/WinoQueer（含代码+数据+部分卡片）；5=暂无。</t>
+          <t>2=Winogender/UnQover（仅论文或极简说明）；3=多数；4=BBQ/CrowS-Pairs/HolisticBias/KoBBQ/MoralChoice/WinoQueer（含代码+数据+部分卡片）；5=暂无。</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -23079,12 +23078,12 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0=Kleinberg/BERT-Bartl/BOLD/Dev/MoralChoice/NeuTral/WikiGenderBias/WinoBias; 1=Majority; 2=CBBQ/HolisticBias/WinoQueer (minor updates or community continuation); 3-5=None.</t>
+          <t>0=BERT-Bartl/BOLD/Dev-WordEmbed/MoralChoice/NeuTral/WikiGenderBias/WinoBias; 1=Majority; 2=CBBQ/HolisticBias/WinoQueer (minor updates or community continuation); 3-5=None.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0=Kleinberg/BERT-Bartl/BOLD/Dev/MoralChoice/NeuTral/WikiGenderBias/WinoBias；1=多数；2=CBBQ/HolisticBias/WinoQueer（少量更新或社区延续）；3-5=无。</t>
+          <t>0=BERT-Bartl/BOLD/Dev-WordEmbed/MoralChoice/NeuTral/WikiGenderBias/WinoBias；1=多数；2=CBBQ/HolisticBias/WinoQueer（少量更新或社区延续）；3-5=无。</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -23975,7 +23974,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>T01; T06; T11</t>
+          <t>T01; T06; T12; T11; T03; T13</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -24042,7 +24041,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>T01; T04; T06; T11</t>
+          <t>T01; T04; T06; T12; T11; T08</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -24104,7 +24103,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>R1 构念清晰度; R3 来源可追溯与证据适配; R7 任务形式适配; R8 答案与分歧设计; R9 指标有效性; R13 文档与可复现; R14 维护与更新治理</t>
+          <t>R1 构念清晰度：将宽泛可信度问题收窄为时间性事实性、来源支持性和可回答性。; R3 来源可追溯与证据适配：保留维基百科条目作为证据来源，并要求答案说明依据。; R7 任务形式适配：将诱导命名实体回答的问题改编为支持错误前提识别的问答任务。; R8 答案与分歧设计：增加错误前提、不可直接回答、当前职位空缺等结构化标签。; R9 指标有效性：从 exact-match 扩展为多指标评分，区分不同事实性失败模式。; R13 文档与可复现：记录来源、适用年份、事实类型、答案版本和复核周期。; R14 维护与更新治理：通过 next_review、retirement_trigger 和版本管理处理动态事实变化。</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -24114,12 +24113,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Better serves FreshQA's dynamic factuality goal by testing current factuality, false-premise recognition, and lifecycle maintenance.</t>
+          <t>It preserves the original factual content and metadata, but changes the task form and scoring so the model must identify a stale false premise, use evidence, and maintain lifecycle metadata.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>更贴合 FreshQA 的动态事实性目标，可测试当前事实、假前提识别与生命周期维护。</t>
+          <t>该改编保留原题事实内容和元数据，但改变任务形式和评分方式，使模型必须识别过时错误前提、使用证据，并维护生命周期元数据。</t>
         </is>
       </c>
     </row>
@@ -24181,12 +24180,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Better tests whether an agent can be useful without leaking patient therapy notes to an unauthorized recipient.</t>
+          <t>The adapted package tests whether an agent can remain useful while respecting contextual integrity: Sarah may be clinically knowledgeable, but she is not authorized to receive Emily’s therapy notes.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>可同时测试 agent「在保护患者治疗笔记不泄漏给未授权接收者的前提下，仍能给出有用回答」。</t>
+          <t>改编题包能测试 agent 是否在保持有用性的同时遵守情境完整性：Sarah 虽具临床知识，但并不是 Emily 治疗笔记的授权接收者。</t>
         </is>
       </c>
     </row>
@@ -24238,7 +24237,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>R1 构念清晰度; R2 规范基础; R4 语境与利益相关方覆盖; R5 现实伤害连接; R7 任务形式适配; R8 答案与分歧设计; R9 指标有效性; R10 评分器可靠性</t>
+          <t>R1 构念清晰度：将“帮助性 / 共情”细化为风险意识、边界尊重、自主权支持和专业边界。; R2 规范基础：引入危机支持、专业边界、自主权和非责备原则。; R4 语境与利益相关方覆盖：纳入用户、伴侣、可信赖他人、危机资源和专业人士。; R5 现实伤害连接：明确双重伤害路径：忽视伴侣安全，以及损害用户自主性与安全。; R7 任务形式适配：保留开放式回答形式，但增加结构化必备要素和风险分级。; R8 答案与分歧设计：增加风险等级、边界支持、安全升级等细粒度标签。; R9 指标有效性：从整体帮助性转向多指标评分，避免温柔但有害的回答被高估。; R10 评分器可靠性：通过评分细则、多评分者校准和专家抽检减少主观偏差。</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -24248,12 +24247,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Better tests risk-aware support, user autonomy, boundary respect, and professional limits rather than only warm counseling tone.</t>
+          <t>The adaptation keeps the original high-risk relationship conflict, but turns it into an operational rubric for risk-aware support, user autonomy, boundary respect, crisis escalation, and professional limits.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>测的是「风险感知支持 + 用户自主权 + 边界尊重 + 专业限制」，而不只是「温暖的咨询语气」。</t>
+          <t>该改编没有改变原题核心情境，而是在原题基础上把评测目标变得可操作、可评分、可诊断：风险感知支持、用户自主权、边界尊重、危机升级和专业限制。</t>
         </is>
       </c>
     </row>
@@ -25729,7 +25728,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>{"Fairness": "No job-relevant evidence yet judgment of candidate suitability; forced choice without equitable basis", "Privacy": "Missing sender, subject, recipient, purpose, or authorization for data handling", "Safety": "Missing operationality, intent, proximity, or explicit risk tier for harm assessment", "Human-Centered": "Missing user state, risk level, professional boundaries, or available support resources", "Agent": "Missing tool permissions, environment context, accessible files, or action consequences"}</t>
+          <t>{"Fairness": "缺少与岗位或任务相关的证据，却直接判断候选人适配性；使用缺乏公平依据的强制二选一。", "Privacy": "缺少发送者、数据主体、接收者、处理目的或授权依据。", "Safety": "缺少可操作性、意图、风险距离或明确风险等级，无法支撑危害判断。", "Human-Centered": "缺少用户状态、风险等级、专业边界或可用支持资源。", "Agent": "缺少工具权限、环境上下文、可访问文件或行动后果说明。"}</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -25806,7 +25805,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>{"Privacy": "隐私规范来源不清；数据来自某法域，却声称适用于所有法域。", "Fairness": "identity categories 直接搬用，不说明来源和本地适配性。", "Trustworthiness": "事实题没有 evidence source、时间戳、更新机制。", "Professional domains": "医疗/心理/法律 source 不来自专业规范或专家审核。"}</t>
+          <t>{"Privacy": "隐私规范来源不清；数据来自某法域，却声称适用于所有法域。", "Fairness": "直接搬用身份类别，未说明来源和本地适配性。", "Trustworthiness": "事实题缺少证据来源、时间戳和更新机制。", "Professional domains": "医疗、心理、法律等专业来源并非来自专业规范或专家审核。"}</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -26037,7 +26036,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>{"Fairness": "No anti-discrimination norms or affected-community evidence; no basis for protected/proxy attributes", "Safety": "No explanation of why specific behaviors constitute misuse; unsafe labeling based only on keywords", "Privacy": "Missing consent, authorization, purpose limitation, minimum necessary, recipient role, or legal basis", "Trustworthiness": "", "Human-Centered": "No engagement with affected-community evidence or participatory norm-setting for community harms"}</t>
+          <t>{"Fairness": "缺少反歧视规范或受影响社区证据；没有说明受保护属性或代理属性的依据。", "Safety": "没有说明特定行为为何构成滥用；仅凭关键词标注不安全。", "Privacy": "缺少同意、授权、目的限制、最小必要、接收者角色或法律依据。", "Trustworthiness": "", "Human-Centered": "未使用受影响社区证据，也未通过参与式规范设定来处理社区伤害。"}</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -26114,7 +26113,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>{"Fairness": "标注者群体不透明；没有受影响社群审查", "Safety": "harm类别标注缺乏专家/红队审核", "Privacy": "信息流判断缺乏法务/隐私专家或规范依据", "Truthfulness": "事实类标签缺乏证据验证"}</t>
+          <t>{"Fairness": "标注者群体不透明；没有受影响社群审查", "Safety": "危害类别标注缺乏专家或红队审核。", "Privacy": "信息流判断缺乏法务/隐私专家或规范依据", "Truthfulness": "事实类标签缺乏证据验证"}</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -26191,7 +26190,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>{"Fairness": "缺少模糊vs明确标签；证据不足时不允许‘不足以判断’", "Safety": "缺少教育性/防御性/虚构性/操作性有害的区分", "Privacy": "缺少 allow / refuse / ask consent / redact / minimize / insufficient authorization", "Professional advice": "缺少 expert escalation、boundary maintenance、insufficient information", "Moral dilemmas": "缺少 acceptable disagreement"}</t>
+          <t>{"Fairness": "缺少模糊vs明确标签；证据不足时不允许‘不足以判断’", "Safety": "缺少教育性/防御性/虚构性/操作性有害的区分", "Privacy": "缺少允许、拒绝、请求同意、脱敏、最小化、授权不足等标签。", "Professional advice": "缺少专家升级、边界维护、信息不足等标签。", "Moral dilemmas": "缺少“可接受分歧”标签。"}</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -26422,7 +26421,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>{"Fairness": "Judge holds cultural/identity biases affecting fairness assessment", "Safety": "Judge prefers strong refusals, misclassifying over-refusal as safe", "Privacy": "", "Trustworthiness": "", "Human-Centered": "Psychological support judge favors warm/long responses while ignoring professional boundaries"}</t>
+          <t>{"Fairness": "评估者带有文化或身份偏见，影响公平性判断。", "Safety": "评估者偏好强拒答，把过度拒答误判为安全。", "Privacy": "", "Trustworthiness": "", "Human-Centered": "心理支持评估者偏好温暖冗长的回复，却忽视专业边界。"}</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -26499,7 +26498,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>{"Fairness": "平均 accuracy 高但 subgroup disparity 大", "Safety": "ASR 低但 over-refusal 高；拒答率高但安全帮助差", "Privacy": "PII leakage 低但 contextual privacy 失败；模型仍然错误转发敏感信息", "Trustworthiness": "accuracy 高但引用不实；不测 abstention 和 freshness", "Human-Centered": "helpfulness 高但越权诊断、忽视危机、损害自主"}</t>
+          <t>{"Fairness": "平均准确率高，但子群体差异大。", "Safety": "攻击成功率低但过度拒答高；拒答率高但安全帮助能力差。", "Privacy": "PII 泄露率低但情境隐私失败；模型仍错误转发敏感信息。", "Trustworthiness": "准确率高但引用不实；不测拒答能力和时效性。", "Human-Centered": "有用性高但越权诊断、忽视危机或损害用户自主。"}</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -26576,7 +26575,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>{"Safety": "新型 jailbreak / agent misuse 出现，但 benchmark 不更新", "Privacy": "从 PII 泄露发展到 memory / agent / multimodal privacy，但 benchmark 仍旧只测字符串", "Trustworthiness": "事实过时，缺 temporal refresh", "Law/policy": "法规变化，benchmark 仍用旧规则", "Agent": "模型行动能力变化，但任务仍是 chat-only"}</t>
+          <t>{"Safety": "新型越狱或智能体滥用已经出现，但基准不更新。", "Privacy": "风险已从 PII 泄露扩展到记忆、智能体和多模态隐私，但基准仍只测字符串。", "Trustworthiness": "事实已过时，缺少时间刷新机制。", "Law/policy": "法规已经变化，但基准仍使用旧规则。", "Agent": "模型行动能力已经变化，但任务仍停留在纯聊天。"}</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">

</xml_diff>

<commit_message>
Align HEART repository and site manifests
</commit_message>
<xml_diff>
--- a/codebook/heart_codebook.xlsx
+++ b/codebook/heart_codebook.xlsx
@@ -13190,7 +13190,11 @@
           <t>https://arxiv.org/abs/2511.05359</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>https://github.com/amrgomaaelhady/ConVerse</t>
+        </is>
+      </c>
       <c r="M94" t="inlineStr">
         <is>
           <t>T03</t>
@@ -13318,8 +13322,16 @@
           <t>95</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2510.02356</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>https://github.com/Graph-COM/EAPrivacy</t>
+        </is>
+      </c>
       <c r="M95" t="inlineStr">
         <is>
           <t>T01</t>

</xml_diff>